<commit_message>
Extend Case Study to Scenarios
</commit_message>
<xml_diff>
--- a/data/fullyear-resilience/Global_Parameters.xlsx
+++ b/data/fullyear-resilience/Global_Parameters.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr codeName="DieseArbeitsmappe" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Simon Malacek\Code\LEGO-Pyomo\data\mini-example-resilience\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Simon Malacek\Code\LEGO-Pyomo\data\fullyear-resilience\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ACB93022-127A-4E4D-8402-A0B72AA53D8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9909969C-A935-4A36-A5A1-6D81EE71B873}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="851" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="95880" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="851" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Global Parameters" sheetId="121" r:id="rId1"/>
@@ -1146,7 +1146,7 @@
         <v>45</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>1</v>
+        <v>47</v>
       </c>
       <c r="E24" s="1" t="s">
         <v>46</v>
@@ -1291,6 +1291,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101004934E3CB1C58BA43BC6E229E2BF20201" ma:contentTypeVersion="4" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="e33ccc94e63df24f58cb47229b46e190">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="87003a75-b64f-4b22-bf19-aa30740e3d46" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0f0f7a5bb162b669de9ce8ff8278c29f" ns2:_="">
     <xsd:import namespace="87003a75-b64f-4b22-bf19-aa30740e3d46"/>
@@ -1436,22 +1451,31 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0155F7A0-74CD-4575-8C0B-A34C113F80FE}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="87003a75-b64f-4b22-bf19-aa30740e3d46"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{13778B2C-CE05-4B32-8196-2F381FEAC95A}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{773946F7-566C-458F-95C9-79B0CCE20E87}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1467,28 +1491,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0155F7A0-74CD-4575-8C0B-A34C113F80FE}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="87003a75-b64f-4b22-bf19-aa30740e3d46"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{13778B2C-CE05-4B32-8196-2F381FEAC95A}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Switch to gurobi persistent
</commit_message>
<xml_diff>
--- a/data/fullyear-resilience/Global_Parameters.xlsx
+++ b/data/fullyear-resilience/Global_Parameters.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Simon Malacek\Code\LEGO-Pyomo\data\fullyear-resilience\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7015F3F-CC3E-47D6-BBA4-4644F4D7C742}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{203C042F-C490-4A07-8EFF-A2E40464950F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="851" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="851" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Global Parameters" sheetId="121" r:id="rId1"/>
@@ -210,9 +210,6 @@
     <t>No</t>
   </si>
   <si>
-    <t>gurobi</t>
-  </si>
-  <si>
     <t>Module Selection</t>
   </si>
   <si>
@@ -235,6 +232,9 @@
   </si>
   <si>
     <t>critial_load_factor</t>
+  </si>
+  <si>
+    <t>gurobi_persistent</t>
   </si>
 </sst>
 </file>
@@ -910,7 +910,7 @@
         <v>40</v>
       </c>
       <c r="C2" s="18" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="3" spans="2:8" s="4" customFormat="1" ht="26.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -950,7 +950,7 @@
         <v>23</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
       <c r="E5" s="11" t="s">
         <v>24</v>
@@ -1166,7 +1166,7 @@
     </row>
     <row r="25" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B25" s="3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C25" s="9">
         <v>48</v>
@@ -1186,7 +1186,7 @@
     </row>
     <row r="26" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B26" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C26" s="9">
         <v>1</v>
@@ -1194,7 +1194,7 @@
     </row>
     <row r="27" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B27" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C27" s="9">
         <v>0.35</v>
@@ -1203,7 +1203,7 @@
     <row r="29" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="7"/>
       <c r="B29" s="7" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C29" s="7"/>
       <c r="D29" s="7"/>
@@ -1218,7 +1218,7 @@
     </row>
     <row r="30" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B30" s="5" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C30" s="1" t="s">
         <v>13</v>
@@ -1226,13 +1226,13 @@
     </row>
     <row r="31" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B31" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C31" s="6" t="s">
         <v>1</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="G31" s="1" t="s">
         <v>8</v>
@@ -1313,6 +1313,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101004934E3CB1C58BA43BC6E229E2BF20201" ma:contentTypeVersion="4" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="e33ccc94e63df24f58cb47229b46e190">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="87003a75-b64f-4b22-bf19-aa30740e3d46" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0f0f7a5bb162b669de9ce8ff8278c29f" ns2:_="">
     <xsd:import namespace="87003a75-b64f-4b22-bf19-aa30740e3d46"/>
@@ -1458,22 +1473,31 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0155F7A0-74CD-4575-8C0B-A34C113F80FE}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="87003a75-b64f-4b22-bf19-aa30740e3d46"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{13778B2C-CE05-4B32-8196-2F381FEAC95A}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{773946F7-566C-458F-95C9-79B0CCE20E87}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1489,28 +1513,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{13778B2C-CE05-4B32-8196-2F381FEAC95A}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0155F7A0-74CD-4575-8C0B-A34C113F80FE}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="87003a75-b64f-4b22-bf19-aa30740e3d46"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>